<commit_message>
Updated data in the elec, fuels, and trans sector
</commit_message>
<xml_diff>
--- a/InputData/elec/PTCF/Peak Time Capacity Factors.xlsx
+++ b/InputData/elec/PTCF/Peak Time Capacity Factors.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10526"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-brazil-cpl/InputData/elec/PTCF/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saido\Documents\eps-brazil-cpl\InputData\elec\PTCF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AD70AB1-C186-E241-9604-77C856CF0DAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="765" windowWidth="34200" windowHeight="21375" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="12" r:id="rId1"/>
@@ -25,7 +24,7 @@
   <definedNames>
     <definedName name="LocalAreaOptions">[1]Lists!$B$11:$B$21</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -216,7 +215,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
@@ -404,13 +403,13 @@
     </xf>
   </cellXfs>
   <cellStyles count="7">
-    <cellStyle name="Body: normal cell" xfId="5" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
-    <cellStyle name="Font: Calibri, 9pt regular" xfId="2" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
-    <cellStyle name="Header: bottom row" xfId="4" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
+    <cellStyle name="Body: normal cell" xfId="5"/>
+    <cellStyle name="Font: Calibri, 9pt regular" xfId="2"/>
+    <cellStyle name="Header: bottom row" xfId="4"/>
+    <cellStyle name="Lien hypertexte" xfId="6" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 6" xfId="1" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
-    <cellStyle name="Table title" xfId="3" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
+    <cellStyle name="Normal 6" xfId="1"/>
+    <cellStyle name="Table title" xfId="3"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -445,7 +444,7 @@
         <xdr:cNvPr id="2" name="Imagem 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{54DC3BFC-0017-45C7-81E6-95668194F06A}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{54DC3BFC-0017-45C7-81E6-95668194F06A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -493,7 +492,7 @@
         <xdr:cNvPr id="4" name="Imagem 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5479D61E-CBCD-4367-ADC0-AD27C27541AD}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{5479D61E-CBCD-4367-ADC0-AD27C27541AD}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -541,7 +540,7 @@
         <xdr:cNvPr id="2" name="Imagem 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BE29AA68-5D54-40DD-B30D-22E7786AC7E5}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{BE29AA68-5D54-40DD-B30D-22E7786AC7E5}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -571,7 +570,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Information"/>
@@ -907,28 +906,28 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H38"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.6640625" customWidth="1"/>
-    <col min="2" max="2" width="134.1640625" customWidth="1"/>
-    <col min="3" max="3" width="8.83203125" style="12"/>
-    <col min="5" max="5" width="49.6640625" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="37.83203125" customWidth="1"/>
-    <col min="8" max="8" width="47.6640625" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" customWidth="1"/>
+    <col min="2" max="2" width="134.140625" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" style="12"/>
+    <col min="5" max="5" width="49.7109375" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" customWidth="1"/>
+    <col min="7" max="7" width="37.85546875" customWidth="1"/>
+    <col min="8" max="8" width="47.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="G2" s="5"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
@@ -941,7 +940,7 @@
       <c r="E3" s="1"/>
       <c r="H3" s="1"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>42</v>
       </c>
@@ -949,17 +948,17 @@
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B5" s="5">
         <v>2019</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B6" s="13" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>44</v>
       </c>
@@ -970,45 +969,45 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H12" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="E13" s="11"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
     </row>
-    <row r="20" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F20" s="2"/>
     </row>
-    <row r="21" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F21" s="6"/>
     </row>
-    <row r="37" spans="1:2" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="38" spans="1:2" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>10</v>
       </c>
@@ -1018,12 +1017,12 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A38" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A38">
       <formula1>"Summer, Winter"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="B6" r:id="rId1" xr:uid="{73EF5FC9-A1E9-4C67-ACDD-25478EAF3849}"/>
+    <hyperlink ref="B6" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>
@@ -1031,15 +1030,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A39FA55C-C114-4DDD-A927-0B05BD7F912E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.33203125" customWidth="1"/>
-    <col min="2" max="2" width="12.5" customWidth="1"/>
+    <col min="1" max="1" width="26.28515625" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>23</v>
       </c>
@@ -1077,7 +1076,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>21</v>
       </c>
@@ -1118,7 +1117,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>36</v>
       </c>
@@ -1159,7 +1158,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>35</v>
       </c>
@@ -1200,7 +1199,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="5" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B5" s="8">
         <f>0.66666*B4+0.33333*B3</f>
         <v>0.38332949999999999</v>
@@ -1250,7 +1249,7 @@
         <v>0.38332949999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B6" s="8">
         <f>B5*B2</f>
         <v>0.14566520999999999</v>
@@ -1304,7 +1303,7 @@
         <v>0.16515112624999997</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="N7">
         <v>1</v>
       </c>
@@ -1317,15 +1316,15 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{484651EB-36A3-4482-99E0-8CBE9CDDEDA3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:P23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="14" max="14" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1" t="s">
@@ -1365,7 +1364,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
@@ -1406,7 +1405,7 @@
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>36</v>
       </c>
@@ -1447,7 +1446,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>35</v>
       </c>
@@ -1488,7 +1487,7 @@
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="5" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="D5" s="8">
         <f>0.66666*D4+0.33333*D3</f>
         <v>0.3933294</v>
@@ -1539,7 +1538,7 @@
       </c>
       <c r="P5" s="8"/>
     </row>
-    <row r="6" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="D6" s="8">
         <f>D5*D2</f>
         <v>0.18093152400000001</v>
@@ -1593,7 +1592,7 @@
         <v>0.24606142824999999</v>
       </c>
     </row>
-    <row r="20" spans="13:14" x14ac:dyDescent="0.2">
+    <row r="20" spans="13:14" x14ac:dyDescent="0.25">
       <c r="M20" t="s">
         <v>54</v>
       </c>
@@ -1601,7 +1600,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="21" spans="13:14" x14ac:dyDescent="0.2">
+    <row r="21" spans="13:14" x14ac:dyDescent="0.25">
       <c r="M21" t="s">
         <v>52</v>
       </c>
@@ -1610,12 +1609,12 @@
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="22" spans="13:14" x14ac:dyDescent="0.2">
+    <row r="22" spans="13:14" x14ac:dyDescent="0.25">
       <c r="M22" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="23" spans="13:14" x14ac:dyDescent="0.2">
+    <row r="23" spans="13:14" x14ac:dyDescent="0.25">
       <c r="M23" t="s">
         <v>52</v>
       </c>
@@ -1630,11 +1629,11 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{214BA780-13B0-4C49-B4ED-7A4C1E735737}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>23</v>
       </c>
@@ -1672,7 +1671,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>37</v>
       </c>
@@ -1713,7 +1712,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3">
         <v>0.25</v>
@@ -1752,7 +1751,7 @@
         <v>0.26</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="8">
         <f t="shared" ref="B4:M4" si="0">AVERAGE(B2:B3)</f>
@@ -1807,7 +1806,7 @@
         <v>0.25166666666666671</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -1823,7 +1822,7 @@
       <c r="M5" s="8"/>
       <c r="N5" s="8"/>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
     </row>
   </sheetData>
@@ -1833,18 +1832,18 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.1640625" customWidth="1"/>
+    <col min="1" max="1" width="24.140625" customWidth="1"/>
     <col min="2" max="3" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
         <v>49</v>
       </c>
@@ -1855,7 +1854,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1867,19 +1866,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="3">
-        <v>0.25</v>
+        <v>0.65</v>
       </c>
       <c r="C3" s="3">
         <f t="shared" ref="C3:C17" si="0">B3</f>
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -1891,7 +1890,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -1903,7 +1902,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -1916,7 +1915,7 @@
         <v>0.16515112624999997</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1929,7 +1928,7 @@
         <v>0.25166666666666671</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -1941,7 +1940,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -1954,7 +1953,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -1966,7 +1965,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -1978,7 +1977,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>0</v>
       </c>
@@ -1990,7 +1989,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -2003,7 +2002,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -2016,7 +2015,7 @@
         <v>0.24606142824999999</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -2029,7 +2028,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>18</v>
       </c>
@@ -2042,7 +2041,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>19</v>
       </c>

</xml_diff>

<commit_message>
Updated BECF, PTCF, and SYC
</commit_message>
<xml_diff>
--- a/InputData/elec/PTCF/Peak Time Capacity Factors.xlsx
+++ b/InputData/elec/PTCF/Peak Time Capacity Factors.xlsx
@@ -9,17 +9,18 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="765" windowWidth="34200" windowHeight="21375" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="765" windowWidth="34200" windowHeight="21375" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="12" r:id="rId1"/>
     <sheet name="Onshore wind" sheetId="42" r:id="rId2"/>
     <sheet name="Offshore wind" sheetId="43" r:id="rId3"/>
     <sheet name="Solar PV" sheetId="44" r:id="rId4"/>
-    <sheet name="PTCF" sheetId="21" r:id="rId5"/>
+    <sheet name="Brazil" sheetId="45" r:id="rId5"/>
+    <sheet name="PTCF" sheetId="21" r:id="rId6"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId6"/>
+    <externalReference r:id="rId7"/>
   </externalReferences>
   <definedNames>
     <definedName name="LocalAreaOptions">[1]Lists!$B$11:$B$21</definedName>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="63">
   <si>
     <t>natural gas nonpeaker</t>
   </si>
@@ -210,6 +211,27 @@
   </si>
   <si>
     <t>Other</t>
+  </si>
+  <si>
+    <t>Calibrated</t>
+  </si>
+  <si>
+    <t>Capacity Factor</t>
+  </si>
+  <si>
+    <t>USA</t>
+  </si>
+  <si>
+    <t>New - BR</t>
+  </si>
+  <si>
+    <t>solar PV</t>
+  </si>
+  <si>
+    <t>geothermal</t>
+  </si>
+  <si>
+    <t>natural gas peaker</t>
   </si>
 </sst>
 </file>
@@ -220,7 +242,7 @@
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -288,8 +310,27 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -314,8 +355,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -356,6 +409,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFC5C2C2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFC5C2C2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFC5C2C2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFC5C2C2"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -372,7 +440,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -401,6 +469,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Body: normal cell" xfId="5"/>
@@ -444,7 +522,7 @@
         <xdr:cNvPr id="2" name="Imagem 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{54DC3BFC-0017-45C7-81E6-95668194F06A}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{54DC3BFC-0017-45C7-81E6-95668194F06A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -492,7 +570,7 @@
         <xdr:cNvPr id="4" name="Imagem 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{5479D61E-CBCD-4367-ADC0-AD27C27541AD}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5479D61E-CBCD-4367-ADC0-AD27C27541AD}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -540,7 +618,7 @@
         <xdr:cNvPr id="2" name="Imagem 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{BE29AA68-5D54-40DD-B30D-22E7786AC7E5}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BE29AA68-5D54-40DD-B30D-22E7786AC7E5}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1833,6 +1911,254 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="D1" s="17" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="19">
+        <v>0.4</v>
+      </c>
+      <c r="C2" s="20">
+        <v>0.48362856194521098</v>
+      </c>
+      <c r="D2" s="20">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="19">
+        <v>0.7</v>
+      </c>
+      <c r="C3" s="20">
+        <v>0.627</v>
+      </c>
+      <c r="D3" s="20">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="19">
+        <v>0.8</v>
+      </c>
+      <c r="C4" s="20">
+        <v>0.92400000000000004</v>
+      </c>
+      <c r="D4" s="20">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="19">
+        <v>0.37</v>
+      </c>
+      <c r="C5" s="20">
+        <v>0.44769999999999999</v>
+      </c>
+      <c r="D5" s="20">
+        <v>0.37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="21" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="19">
+        <v>0.35</v>
+      </c>
+      <c r="C6" s="20">
+        <v>0.38662000000000002</v>
+      </c>
+      <c r="D6" s="20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="B7" s="19">
+        <v>0.215</v>
+      </c>
+      <c r="C7" s="20">
+        <v>0.2514666287530456</v>
+      </c>
+      <c r="D7" s="20">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" s="19">
+        <v>0.215</v>
+      </c>
+      <c r="C8" s="20">
+        <v>0.58933333333333326</v>
+      </c>
+      <c r="D8" s="20">
+        <v>0.59</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="19">
+        <v>0.5</v>
+      </c>
+      <c r="C9" s="20">
+        <v>0.6875</v>
+      </c>
+      <c r="D9" s="20">
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="19">
+        <v>0.82</v>
+      </c>
+      <c r="C10" s="20">
+        <v>0.7601</v>
+      </c>
+      <c r="D10" s="20">
+        <v>0.76</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" s="19">
+        <v>0.15</v>
+      </c>
+      <c r="C11" s="20">
+        <v>6.1966666666666677E-2</v>
+      </c>
+      <c r="D11" s="20">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" s="19">
+        <v>0.3</v>
+      </c>
+      <c r="C12" s="20">
+        <v>0.14630000000000001</v>
+      </c>
+      <c r="D12" s="20">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="19">
+        <v>0.4</v>
+      </c>
+      <c r="C13" s="20">
+        <v>0.83400921942536133</v>
+      </c>
+      <c r="D13" s="20">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="19">
+        <v>0.6</v>
+      </c>
+      <c r="C14" s="20">
+        <v>0.48769523684708904</v>
+      </c>
+      <c r="D14" s="20">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="19">
+        <v>0.15</v>
+      </c>
+      <c r="C15" s="20">
+        <v>6.1966666666666677E-2</v>
+      </c>
+      <c r="D15" s="20">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="19">
+        <v>0.15</v>
+      </c>
+      <c r="C16" s="20">
+        <v>6.1966666666666677E-2</v>
+      </c>
+      <c r="D16" s="20">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="19">
+        <v>0.5</v>
+      </c>
+      <c r="C17" s="20">
+        <v>0.71060000000000012</v>
+      </c>
+      <c r="D17" s="20">
+        <v>0.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
@@ -2046,7 +2372,6 @@
         <v>19</v>
       </c>
       <c r="B17" s="3">
-        <f>B9</f>
         <v>0.4</v>
       </c>
       <c r="C17" s="3">

</xml_diff>